<commit_message>
CARLA-5 final documents re-check
</commit_message>
<xml_diff>
--- a/rmonize/data_proc_elem/CARLA_P1_FFQ_Information.xlsx
+++ b/rmonize/data_proc_elem/CARLA_P1_FFQ_Information.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20394"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\schwarz-f\Desktop\use-cases-harmonisation\rmonize\data_proc_elem\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\schwarz-f\Desktop\CARLA\use-cases-harmonisation\rmonize\data_proc_elem\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BCC2CAEE-F408-42EA-8E93-C61C03DC48B5}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9D09575-2CF1-4D89-B9E6-56251D4C4750}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="10125" xr2:uid="{BE203D1B-CAC6-41E8-A7D9-4743C8A656B5}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BE203D1B-CAC6-41E8-A7D9-4743C8A656B5}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -20,12 +20,15 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="99">
   <si>
     <t>Name</t>
   </si>
@@ -144,9 +147,6 @@
     <t>BREAKF_CEREALS_0604</t>
   </si>
   <si>
-    <t>SALT_BISCUIT_0605</t>
-  </si>
-  <si>
     <t>DOUGH_PASTRY_0606</t>
   </si>
   <si>
@@ -165,9 +165,6 @@
     <t>PORK_070103</t>
   </si>
   <si>
-    <t>MUTTON_LAMB_070104</t>
-  </si>
-  <si>
     <t>POULTRY_0702</t>
   </si>
   <si>
@@ -177,9 +174,6 @@
     <t>CHICKEN_070201</t>
   </si>
   <si>
-    <t>RABBIT_070205</t>
-  </si>
-  <si>
     <t>PROCMEAT_0704</t>
   </si>
   <si>
@@ -267,9 +261,6 @@
     <t>HERBALTEA_130303</t>
   </si>
   <si>
-    <t>COFFEE_IMITATE_130304</t>
-  </si>
-  <si>
     <t>WATER_1304</t>
   </si>
   <si>
@@ -310,9 +301,6 @@
   </si>
   <si>
     <t>HERBS_SPICES_1503</t>
-  </si>
-  <si>
-    <t>CONDIMENTS_1504</t>
   </si>
   <si>
     <t>SOUP_BOUILLON_16</t>
@@ -392,9 +380,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 – 2022-Design">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 – 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -432,7 +420,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 – 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -538,7 +526,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 – 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -680,7 +668,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -688,7 +676,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1510091C-455E-4711-A209-8BD9D6DEB1E6}">
-  <dimension ref="A1:D101"/>
+  <dimension ref="A1:D96"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.140625" bestFit="1" customWidth="1"/>
@@ -1092,7 +1080,7 @@
         <v>6</v>
       </c>
       <c r="C37">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
@@ -1100,10 +1088,7 @@
         <v>40</v>
       </c>
       <c r="B38">
-        <v>6</v>
-      </c>
-      <c r="C38">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
@@ -1113,6 +1098,9 @@
       <c r="B39">
         <v>7</v>
       </c>
+      <c r="C39">
+        <v>1</v>
+      </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
@@ -1124,6 +1112,9 @@
       <c r="C40">
         <v>1</v>
       </c>
+      <c r="D40">
+        <v>1</v>
+      </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
@@ -1136,7 +1127,7 @@
         <v>1</v>
       </c>
       <c r="D41">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
@@ -1150,7 +1141,7 @@
         <v>1</v>
       </c>
       <c r="D42">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
@@ -1161,10 +1152,7 @@
         <v>7</v>
       </c>
       <c r="C43">
-        <v>1</v>
-      </c>
-      <c r="D43">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
@@ -1175,10 +1163,10 @@
         <v>7</v>
       </c>
       <c r="C44">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D44">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
@@ -1191,6 +1179,9 @@
       <c r="C45">
         <v>2</v>
       </c>
+      <c r="D45">
+        <v>1</v>
+      </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
@@ -1200,10 +1191,7 @@
         <v>7</v>
       </c>
       <c r="C46">
-        <v>2</v>
-      </c>
-      <c r="D46">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
@@ -1214,10 +1202,7 @@
         <v>7</v>
       </c>
       <c r="C47">
-        <v>2</v>
-      </c>
-      <c r="D47">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
@@ -1225,95 +1210,92 @@
         <v>50</v>
       </c>
       <c r="B48">
-        <v>7</v>
-      </c>
-      <c r="C48">
-        <v>2</v>
-      </c>
-      <c r="D48">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>51</v>
       </c>
       <c r="B49">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C49">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>52</v>
       </c>
       <c r="B50">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C50">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>53</v>
       </c>
       <c r="B51">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>54</v>
       </c>
       <c r="B52">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C52">
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>55</v>
       </c>
       <c r="B53">
-        <v>8</v>
-      </c>
-      <c r="C53">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>56</v>
       </c>
       <c r="B54">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+      <c r="C54">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>57</v>
       </c>
       <c r="B55">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C55">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>58</v>
       </c>
       <c r="B56">
         <v>10</v>
       </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C56">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>59</v>
       </c>
@@ -1321,10 +1303,10 @@
         <v>10</v>
       </c>
       <c r="C57">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>60</v>
       </c>
@@ -1332,51 +1314,51 @@
         <v>10</v>
       </c>
       <c r="C58">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>61</v>
       </c>
       <c r="B59">
-        <v>10</v>
-      </c>
-      <c r="C59">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>62</v>
       </c>
       <c r="B60">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C60">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>63</v>
       </c>
       <c r="B61">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C61">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>64</v>
       </c>
       <c r="B62">
         <v>11</v>
       </c>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C62">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>65</v>
       </c>
@@ -1384,10 +1366,10 @@
         <v>11</v>
       </c>
       <c r="C63">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>66</v>
       </c>
@@ -1395,7 +1377,10 @@
         <v>11</v>
       </c>
       <c r="C64">
-        <v>2</v>
+        <v>5</v>
+      </c>
+      <c r="D64">
+        <v>1</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
@@ -1403,10 +1388,7 @@
         <v>67</v>
       </c>
       <c r="B65">
-        <v>11</v>
-      </c>
-      <c r="C65">
-        <v>3</v>
+        <v>12</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
@@ -1414,10 +1396,10 @@
         <v>68</v>
       </c>
       <c r="B66">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C66">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
@@ -1425,13 +1407,10 @@
         <v>69</v>
       </c>
       <c r="B67">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C67">
-        <v>5</v>
-      </c>
-      <c r="D67">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
@@ -1439,7 +1418,7 @@
         <v>70</v>
       </c>
       <c r="B68">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
@@ -1447,7 +1426,7 @@
         <v>71</v>
       </c>
       <c r="B69">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C69">
         <v>1</v>
@@ -1458,7 +1437,7 @@
         <v>72</v>
       </c>
       <c r="B70">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C70">
         <v>2</v>
@@ -1471,6 +1450,9 @@
       <c r="B71">
         <v>13</v>
       </c>
+      <c r="C71">
+        <v>3</v>
+      </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
@@ -1480,6 +1462,9 @@
         <v>13</v>
       </c>
       <c r="C72">
+        <v>3</v>
+      </c>
+      <c r="D72">
         <v>1</v>
       </c>
     </row>
@@ -1491,6 +1476,9 @@
         <v>13</v>
       </c>
       <c r="C73">
+        <v>3</v>
+      </c>
+      <c r="D73">
         <v>2</v>
       </c>
     </row>
@@ -1504,6 +1492,9 @@
       <c r="C74">
         <v>3</v>
       </c>
+      <c r="D74">
+        <v>3</v>
+      </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
@@ -1513,10 +1504,7 @@
         <v>13</v>
       </c>
       <c r="C75">
-        <v>3</v>
-      </c>
-      <c r="D75">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
@@ -1524,13 +1512,7 @@
         <v>78</v>
       </c>
       <c r="B76">
-        <v>13</v>
-      </c>
-      <c r="C76">
-        <v>3</v>
-      </c>
-      <c r="D76">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
@@ -1538,13 +1520,10 @@
         <v>79</v>
       </c>
       <c r="B77">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C77">
-        <v>3</v>
-      </c>
-      <c r="D77">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
@@ -1552,13 +1531,10 @@
         <v>80</v>
       </c>
       <c r="B78">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C78">
-        <v>3</v>
-      </c>
-      <c r="D78">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
@@ -1566,10 +1542,10 @@
         <v>81</v>
       </c>
       <c r="B79">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C79">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
@@ -1579,6 +1555,9 @@
       <c r="B80">
         <v>14</v>
       </c>
+      <c r="C80">
+        <v>4</v>
+      </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
@@ -1588,7 +1567,7 @@
         <v>14</v>
       </c>
       <c r="C81">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
@@ -1599,7 +1578,7 @@
         <v>14</v>
       </c>
       <c r="C82">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
@@ -1607,10 +1586,7 @@
         <v>85</v>
       </c>
       <c r="B83">
-        <v>14</v>
-      </c>
-      <c r="C83">
-        <v>3</v>
+        <v>15</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
@@ -1618,10 +1594,10 @@
         <v>86</v>
       </c>
       <c r="B84">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C84">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
@@ -1629,10 +1605,13 @@
         <v>87</v>
       </c>
       <c r="B85">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C85">
-        <v>5</v>
+        <v>1</v>
+      </c>
+      <c r="D85">
+        <v>1</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
@@ -1640,10 +1619,13 @@
         <v>88</v>
       </c>
       <c r="B86">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C86">
-        <v>6</v>
+        <v>1</v>
+      </c>
+      <c r="D86">
+        <v>2</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
@@ -1653,6 +1635,12 @@
       <c r="B87">
         <v>15</v>
       </c>
+      <c r="C87">
+        <v>1</v>
+      </c>
+      <c r="D87">
+        <v>3</v>
+      </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
@@ -1662,7 +1650,7 @@
         <v>15</v>
       </c>
       <c r="C88">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
@@ -1670,13 +1658,7 @@
         <v>91</v>
       </c>
       <c r="B89">
-        <v>15</v>
-      </c>
-      <c r="C89">
-        <v>1</v>
-      </c>
-      <c r="D89">
-        <v>1</v>
+        <v>16</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
@@ -1684,13 +1666,10 @@
         <v>92</v>
       </c>
       <c r="B90">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C90">
         <v>1</v>
-      </c>
-      <c r="D90">
-        <v>2</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
@@ -1698,13 +1677,10 @@
         <v>93</v>
       </c>
       <c r="B91">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C91">
-        <v>1</v>
-      </c>
-      <c r="D91">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
@@ -1712,10 +1688,7 @@
         <v>94</v>
       </c>
       <c r="B92">
-        <v>15</v>
-      </c>
-      <c r="C92">
-        <v>3</v>
+        <v>17</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
@@ -1723,10 +1696,10 @@
         <v>95</v>
       </c>
       <c r="B93">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C93">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
@@ -1734,7 +1707,10 @@
         <v>96</v>
       </c>
       <c r="B94">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="C94">
+        <v>1</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
@@ -1742,10 +1718,10 @@
         <v>97</v>
       </c>
       <c r="B95">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C95">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
@@ -1753,64 +1729,12 @@
         <v>98</v>
       </c>
       <c r="B96">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C96">
         <v>2</v>
       </c>
-    </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A97" t="s">
-        <v>99</v>
-      </c>
-      <c r="B97">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A98" t="s">
-        <v>100</v>
-      </c>
-      <c r="B98">
-        <v>17</v>
-      </c>
-      <c r="C98">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A99" t="s">
-        <v>101</v>
-      </c>
-      <c r="B99">
-        <v>17</v>
-      </c>
-      <c r="C99">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A100" t="s">
-        <v>102</v>
-      </c>
-      <c r="B100">
-        <v>17</v>
-      </c>
-      <c r="C100">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A101" t="s">
-        <v>103</v>
-      </c>
-      <c r="B101">
-        <v>17</v>
-      </c>
-      <c r="C101">
-        <v>2</v>
-      </c>
-      <c r="D101">
+      <c r="D96">
         <v>1</v>
       </c>
     </row>

</xml_diff>